<commit_message>
healthy days (winter) updated
</commit_message>
<xml_diff>
--- a/output/tables/table_S3_healthy_days_2.0.xlsx
+++ b/output/tables/table_S3_healthy_days_2.0.xlsx
@@ -1025,7 +1025,16 @@
         <v>106</v>
       </c>
       <c r="I16" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="J16">
+        <v>97.17</v>
+      </c>
+      <c r="K16">
+        <v>84.91</v>
+      </c>
+      <c r="L16">
+        <v>23.58</v>
       </c>
     </row>
     <row r="17">
@@ -1142,7 +1151,16 @@
         <v>106</v>
       </c>
       <c r="I19" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="J19">
+        <v>80.19</v>
+      </c>
+      <c r="K19">
+        <v>54.72</v>
+      </c>
+      <c r="L19">
+        <v>15.09</v>
       </c>
     </row>
     <row r="20">
@@ -1259,7 +1277,16 @@
         <v>106</v>
       </c>
       <c r="I22" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="J22">
+        <v>58.49</v>
+      </c>
+      <c r="K22">
+        <v>36.79</v>
+      </c>
+      <c r="L22">
+        <v>10.38</v>
       </c>
     </row>
     <row r="23">

</xml_diff>